<commit_message>
test run CuongNHHE, no docker container being deployed
</commit_message>
<xml_diff>
--- a/GradeSession_1_Dec/1/StudentsSolution.xlsx
+++ b/GradeSession_1_Dec/1/StudentsSolution.xlsx
@@ -46,10 +46,13 @@
     <x:t>Success</x:t>
   </x:si>
   <x:si>
-    <x:t>01-12-2025 03:15:12</x:t>
-  </x:si>
-  <x:si>
-    <x:t>01-12-2025 03:15:59</x:t>
+    <x:t>0</x:t>
+  </x:si>
+  <x:si>
+    <x:t>02-12-2025 12:32:53</x:t>
+  </x:si>
+  <x:si>
+    <x:t>02-12-2025 12:34:41</x:t>
   </x:si>
   <x:si>
     <x:t>2</x:t>
@@ -58,16 +61,16 @@
     <x:t>dongnvhe172649</x:t>
   </x:si>
   <x:si>
-    <x:t>01-12-2025 03:16:52</x:t>
+    <x:t>Not Run</x:t>
+  </x:si>
+  <x:si>
+    <x:t/>
   </x:si>
   <x:si>
     <x:t>3</x:t>
   </x:si>
   <x:si>
     <x:t>hoangbsthe186345</x:t>
-  </x:si>
-  <x:si>
-    <x:t>01-12-2025 03:17:45</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -456,7 +459,7 @@
     <x:col min="1" max="1" width="3.424911" style="0" customWidth="1"/>
     <x:col min="2" max="2" width="18.139196" style="0" customWidth="1"/>
     <x:col min="3" max="3" width="10.853482" style="0" customWidth="1"/>
-    <x:col min="4" max="4" width="7.853482" style="0" customWidth="1"/>
+    <x:col min="4" max="4" width="8.282054" style="0" customWidth="1"/>
     <x:col min="5" max="5" width="10.567768" style="0" customWidth="1"/>
     <x:col min="6" max="7" width="18.567768" style="0" customWidth="1"/>
   </x:cols>
@@ -498,59 +501,59 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="E2" s="2" t="s">
-        <x:v>7</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F2" s="2" t="s">
-        <x:v>10</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="G2" s="2" t="s">
-        <x:v>11</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:7">
-      <x:c r="A3" s="2" t="s">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="B3" s="2" t="s">
+      <x:c r="A3" s="0" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="C3" s="2" t="s">
+      <x:c r="B3" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="C3" s="0" t="s">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="D3" s="2" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="E3" s="2" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="F3" s="2" t="s">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="G3" s="2" t="s">
-        <x:v>14</x:v>
+      <x:c r="D3" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="E3" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F3" s="0" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="G3" s="0" t="s">
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:7">
-      <x:c r="A4" s="2" t="s">
+      <x:c r="A4" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B4" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="C4" s="0" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="D4" s="0" t="s">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="B4" s="2" t="s">
+      <x:c r="E4" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F4" s="0" t="s">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="C4" s="2" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="D4" s="2" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="E4" s="2" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="F4" s="2" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="G4" s="2" t="s">
-        <x:v>17</x:v>
+      <x:c r="G4" s="0" t="s">
+        <x:v>16</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
test run, minor error
</commit_message>
<xml_diff>
--- a/GradeSession_1_Dec/1/StudentsSolution.xlsx
+++ b/GradeSession_1_Dec/1/StudentsSolution.xlsx
@@ -46,13 +46,10 @@
     <x:t>Success</x:t>
   </x:si>
   <x:si>
-    <x:t>0</x:t>
-  </x:si>
-  <x:si>
-    <x:t>02-12-2025 12:32:53</x:t>
-  </x:si>
-  <x:si>
-    <x:t>02-12-2025 12:34:41</x:t>
+    <x:t>02-12-2025 13:44:58</x:t>
+  </x:si>
+  <x:si>
+    <x:t>02-12-2025 13:46:24</x:t>
   </x:si>
   <x:si>
     <x:t>2</x:t>
@@ -61,16 +58,22 @@
     <x:t>dongnvhe172649</x:t>
   </x:si>
   <x:si>
-    <x:t>Not Run</x:t>
-  </x:si>
-  <x:si>
-    <x:t/>
+    <x:t>02-12-2025 13:46:25</x:t>
+  </x:si>
+  <x:si>
+    <x:t>02-12-2025 13:47:35</x:t>
   </x:si>
   <x:si>
     <x:t>3</x:t>
   </x:si>
   <x:si>
     <x:t>hoangbsthe186345</x:t>
+  </x:si>
+  <x:si>
+    <x:t>02-12-2025 13:47:36</x:t>
+  </x:si>
+  <x:si>
+    <x:t>02-12-2025 13:48:46</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -459,7 +462,7 @@
     <x:col min="1" max="1" width="3.424911" style="0" customWidth="1"/>
     <x:col min="2" max="2" width="18.139196" style="0" customWidth="1"/>
     <x:col min="3" max="3" width="10.853482" style="0" customWidth="1"/>
-    <x:col min="4" max="4" width="8.282054" style="0" customWidth="1"/>
+    <x:col min="4" max="4" width="7.853482" style="0" customWidth="1"/>
     <x:col min="5" max="5" width="10.567768" style="0" customWidth="1"/>
     <x:col min="6" max="7" width="18.567768" style="0" customWidth="1"/>
   </x:cols>
@@ -501,59 +504,59 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="E2" s="2" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="F2" s="2" t="s">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="F2" s="2" t="s">
+      <x:c r="G2" s="2" t="s">
         <x:v>11</x:v>
-      </x:c>
-      <x:c r="G2" s="2" t="s">
-        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:7">
-      <x:c r="A3" s="0" t="s">
+      <x:c r="A3" s="2" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B3" s="2" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="B3" s="0" t="s">
+      <x:c r="C3" s="2" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="D3" s="2" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E3" s="2" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="F3" s="2" t="s">
         <x:v>14</x:v>
       </x:c>
-      <x:c r="C3" s="0" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="D3" s="0" t="s">
+      <x:c r="G3" s="2" t="s">
         <x:v>15</x:v>
-      </x:c>
-      <x:c r="E3" s="0" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="F3" s="0" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="G3" s="0" t="s">
-        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:7">
-      <x:c r="A4" s="0" t="s">
+      <x:c r="A4" s="2" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B4" s="2" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="B4" s="0" t="s">
+      <x:c r="C4" s="2" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="D4" s="2" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E4" s="2" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="F4" s="2" t="s">
         <x:v>18</x:v>
       </x:c>
-      <x:c r="C4" s="0" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="D4" s="0" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="E4" s="0" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="F4" s="0" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="G4" s="0" t="s">
-        <x:v>16</x:v>
+      <x:c r="G4" s="2" t="s">
+        <x:v>19</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
adding sample grading log
</commit_message>
<xml_diff>
--- a/GradeSession_1_Dec/1/StudentsSolution.xlsx
+++ b/GradeSession_1_Dec/1/StudentsSolution.xlsx
@@ -46,10 +46,10 @@
     <x:t>Success</x:t>
   </x:si>
   <x:si>
-    <x:t>02-12-2025 13:44:58</x:t>
-  </x:si>
-  <x:si>
-    <x:t>02-12-2025 13:46:24</x:t>
+    <x:t>02-12-2025 15:50:10</x:t>
+  </x:si>
+  <x:si>
+    <x:t>02-12-2025 15:51:46</x:t>
   </x:si>
   <x:si>
     <x:t>2</x:t>
@@ -58,22 +58,19 @@
     <x:t>dongnvhe172649</x:t>
   </x:si>
   <x:si>
-    <x:t>02-12-2025 13:46:25</x:t>
-  </x:si>
-  <x:si>
-    <x:t>02-12-2025 13:47:35</x:t>
+    <x:t>Not Run</x:t>
+  </x:si>
+  <x:si>
+    <x:t>0</x:t>
+  </x:si>
+  <x:si>
+    <x:t/>
   </x:si>
   <x:si>
     <x:t>3</x:t>
   </x:si>
   <x:si>
     <x:t>hoangbsthe186345</x:t>
-  </x:si>
-  <x:si>
-    <x:t>02-12-2025 13:47:36</x:t>
-  </x:si>
-  <x:si>
-    <x:t>02-12-2025 13:48:46</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -462,7 +459,7 @@
     <x:col min="1" max="1" width="3.424911" style="0" customWidth="1"/>
     <x:col min="2" max="2" width="18.139196" style="0" customWidth="1"/>
     <x:col min="3" max="3" width="10.853482" style="0" customWidth="1"/>
-    <x:col min="4" max="4" width="7.853482" style="0" customWidth="1"/>
+    <x:col min="4" max="4" width="8.282054" style="0" customWidth="1"/>
     <x:col min="5" max="5" width="10.567768" style="0" customWidth="1"/>
     <x:col min="6" max="7" width="18.567768" style="0" customWidth="1"/>
   </x:cols>
@@ -514,49 +511,49 @@
       </x:c>
     </x:row>
     <x:row r="3" spans="1:7">
-      <x:c r="A3" s="2" t="s">
+      <x:c r="A3" s="0" t="s">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="B3" s="2" t="s">
+      <x:c r="B3" s="0" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="C3" s="2" t="s">
+      <x:c r="C3" s="0" t="s">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="D3" s="2" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="E3" s="2" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="F3" s="2" t="s">
+      <x:c r="D3" s="0" t="s">
         <x:v>14</x:v>
       </x:c>
-      <x:c r="G3" s="2" t="s">
+      <x:c r="E3" s="0" t="s">
         <x:v>15</x:v>
+      </x:c>
+      <x:c r="F3" s="0" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="G3" s="0" t="s">
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:7">
-      <x:c r="A4" s="2" t="s">
+      <x:c r="A4" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B4" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="C4" s="0" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="D4" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="E4" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F4" s="0" t="s">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="B4" s="2" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="C4" s="2" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="D4" s="2" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="E4" s="2" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="F4" s="2" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="G4" s="2" t="s">
-        <x:v>19</x:v>
+      <x:c r="G4" s="0" t="s">
+        <x:v>16</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
adding sample log after successful run
</commit_message>
<xml_diff>
--- a/GradeSession_1_Dec/1/StudentsSolution.xlsx
+++ b/GradeSession_1_Dec/1/StudentsSolution.xlsx
@@ -46,10 +46,10 @@
     <x:t>Success</x:t>
   </x:si>
   <x:si>
-    <x:t>02-12-2025 15:50:10</x:t>
-  </x:si>
-  <x:si>
-    <x:t>02-12-2025 15:51:46</x:t>
+    <x:t>02-12-2025 21:01:38</x:t>
+  </x:si>
+  <x:si>
+    <x:t>02-12-2025 21:03:32</x:t>
   </x:si>
   <x:si>
     <x:t>2</x:t>

</xml_diff>